<commit_message>
data: mise à jour contenu liste joueurs Groupe B (-9)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/@Liste GROUPE B-9.xlsx
+++ b/public/data/@Liste GROUPE B-9.xlsx
@@ -1133,7 +1133,7 @@
     <t>MOUSSA</t>
   </si>
   <si>
-    <t>MOHAMED</t>
+    <t>MOHAMED MAMADOU</t>
   </si>
   <si>
     <t>ALESSANDRO DIAZ</t>
@@ -2349,11 +2349,11 @@
     <xf borderId="1" fillId="11" fontId="33" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="31" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="31" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
@@ -9873,7 +9873,7 @@
       <c r="D14" s="100" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="101" t="s">
+      <c r="E14" s="105" t="s">
         <v>365</v>
       </c>
       <c r="F14" s="101" t="s">
@@ -10213,7 +10213,7 @@
         <v>383</v>
       </c>
       <c r="G23" s="44"/>
-      <c r="H23" s="105" t="s">
+      <c r="H23" s="106" t="s">
         <v>71</v>
       </c>
       <c r="I23" s="31"/>
@@ -10317,10 +10317,10 @@
       <c r="D26" s="100" t="s">
         <v>94</v>
       </c>
-      <c r="E26" s="106" t="s">
+      <c r="E26" s="105" t="s">
         <v>388</v>
       </c>
-      <c r="F26" s="106" t="s">
+      <c r="F26" s="105" t="s">
         <v>389</v>
       </c>
       <c r="G26" s="44"/>

</xml_diff>